<commit_message>
feat: added jinja2 variables to the template
</commit_message>
<xml_diff>
--- a/templates/payment_order/payment_order.xlsx
+++ b/templates/payment_order/payment_order.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mariano\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\uta-gestion-ops\templates\payment_order\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>IMPUTACION CONTABLE</t>
   </si>
@@ -115,13 +115,6 @@
   </si>
   <si>
     <t xml:space="preserve">R E T E N C I O N E S </t>
-  </si>
-  <si>
-    <t>1300564/23</t>
-  </si>
-  <si>
-    <t>UNION TRANVIARIOS AUTOMOTOR
-S I N D I C A L</t>
   </si>
   <si>
     <t>SECRETARIO
@@ -139,6 +132,46 @@
     <t>BRAVO
 SERGIO
 PABLO</t>
+  </si>
+  <si>
+    <t>UNION TRANVIARIOS AUTOMOTOR
+{{ account_name }}</t>
+  </si>
+  <si>
+    <t>{{ paymnet_order_id }}</t>
+  </si>
+  <si>
+    <t>{{ payment_order_date }}</t>
+  </si>
+  <si>
+    <t>{{ supplier_name }}</t>
+  </si>
+  <si>
+    <t>{{ invoice_amount }}</t>
+  </si>
+  <si>
+    <t>{{ detail }}</t>
+  </si>
+  <si>
+    <t>{{ witholding_amount }}</t>
+  </si>
+  <si>
+    <t>{{ payment_order_total }}</t>
+  </si>
+  <si>
+    <t>{{ invoice_number }}</t>
+  </si>
+  <si>
+    <t>{{ account_number }}</t>
+  </si>
+  <si>
+    <t>{{ check_number }}</t>
+  </si>
+  <si>
+    <t>{{ issue_date }}</t>
+  </si>
+  <si>
+    <t>{{ due_date }}</t>
   </si>
 </sst>
 </file>
@@ -831,87 +864,55 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -968,53 +969,85 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1412,71 +1445,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="62" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
+      <c r="A1" s="50" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="51"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
       <c r="F1" s="26"/>
     </row>
     <row r="2" spans="1:6" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="64"/>
-      <c r="B2" s="65"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
+      <c r="A2" s="52"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
       <c r="F2" s="4"/>
     </row>
     <row r="3" spans="1:6" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="67" t="s">
+      <c r="A3" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="5">
-        <v>0</v>
+      <c r="B3" s="56"/>
+      <c r="C3" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="57" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="58"/>
+      <c r="C4" s="59" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="61"/>
+    </row>
+    <row r="5" spans="1:6" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="62" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="69" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="70"/>
-      <c r="C4" s="71">
-        <v>0</v>
-      </c>
-      <c r="D4" s="72"/>
-      <c r="E4" s="72"/>
-      <c r="F4" s="73"/>
-    </row>
-    <row r="5" spans="1:6" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="74" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="32"/>
+      <c r="B5" s="63"/>
+      <c r="C5" s="63"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="38"/>
     </row>
     <row r="6" spans="1:6" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="76" t="s">
+      <c r="A6" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="77"/>
-      <c r="C6" s="77"/>
-      <c r="D6" s="78" t="s">
+      <c r="B6" s="65"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="79"/>
+      <c r="E6" s="67"/>
       <c r="F6" s="8" t="s">
         <v>3</v>
       </c>
@@ -1485,139 +1518,139 @@
       <c r="A7" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="60"/>
-      <c r="C7" s="61"/>
-      <c r="D7" s="80"/>
-      <c r="E7" s="80"/>
-      <c r="F7" s="14">
-        <v>0</v>
+      <c r="B7" s="48"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="14" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="43">
-        <v>0</v>
-      </c>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
+      <c r="A8" s="92" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="93"/>
+      <c r="C8" s="93"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
       <c r="F8" s="15"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="45"/>
-      <c r="B9" s="44"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="41"/>
+      <c r="A9" s="94"/>
+      <c r="B9" s="93"/>
+      <c r="C9" s="93"/>
+      <c r="D9" s="89"/>
+      <c r="E9" s="90"/>
       <c r="F9" s="15"/>
     </row>
     <row r="10" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="45"/>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
+      <c r="A10" s="94"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="88"/>
+      <c r="E10" s="88"/>
       <c r="F10" s="16"/>
     </row>
     <row r="11" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="45"/>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
+      <c r="A11" s="94"/>
+      <c r="B11" s="93"/>
+      <c r="C11" s="93"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="88"/>
       <c r="F11" s="16"/>
     </row>
     <row r="12" spans="1:6" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="46"/>
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="42" t="s">
+      <c r="A12" s="95"/>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="91" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="17">
-        <v>0</v>
+      <c r="E12" s="91"/>
+      <c r="F12" s="17" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="81" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="31"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="13">
-        <v>0</v>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="13" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="82" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="34"/>
-      <c r="C14" s="35"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="84"/>
       <c r="D14" s="29"/>
       <c r="E14" s="29"/>
       <c r="F14" s="24"/>
     </row>
     <row r="15" spans="1:6" s="2" customFormat="1" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="53"/>
-      <c r="C15" s="54">
-        <v>0</v>
-      </c>
-      <c r="D15" s="55"/>
-      <c r="E15" s="56"/>
-      <c r="F15" s="57"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="75" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="76"/>
+      <c r="E15" s="77"/>
+      <c r="F15" s="78"/>
     </row>
     <row r="16" spans="1:6" ht="28.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="85" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="58" t="s">
+      <c r="B16" s="86"/>
+      <c r="C16" s="87"/>
+      <c r="D16" s="79" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="59"/>
+      <c r="E16" s="80"/>
       <c r="F16" s="20" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="19">
-        <v>0</v>
+      <c r="B17" s="19" t="s">
+        <v>42</v>
       </c>
       <c r="C17" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="23">
-        <v>0</v>
+      <c r="D17" s="23" t="s">
+        <v>43</v>
       </c>
       <c r="E17" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="22">
-        <v>0</v>
+      <c r="F17" s="22" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="50" t="s">
+      <c r="A18" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="51"/>
-      <c r="C18" s="51"/>
-      <c r="D18" s="48" t="s">
+      <c r="B18" s="72"/>
+      <c r="C18" s="72"/>
+      <c r="D18" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="48"/>
-      <c r="F18" s="49"/>
+      <c r="E18" s="69"/>
+      <c r="F18" s="70"/>
     </row>
     <row r="19" spans="1:6" ht="5.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="10"/>
@@ -1631,29 +1664,29 @@
       <c r="A20" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="81" t="s">
+      <c r="B20" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="82"/>
-      <c r="D20" s="82"/>
-      <c r="E20" s="82"/>
-      <c r="F20" s="83"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="34"/>
     </row>
     <row r="21" spans="1:6" ht="62.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="96" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="92" t="s">
+      <c r="A21" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="45"/>
+      <c r="D21" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="91"/>
-      <c r="D21" s="93" t="s">
-        <v>31</v>
-      </c>
-      <c r="E21" s="95" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" s="94"/>
+      <c r="F21" s="47"/>
     </row>
     <row r="22" spans="1:6" ht="5.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10"/>
@@ -1664,28 +1697,28 @@
       <c r="F22" s="11"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="84" t="s">
+      <c r="A23" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="85"/>
-      <c r="C23" s="85"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="32"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="38"/>
     </row>
     <row r="24" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="86" t="s">
+      <c r="A24" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B24" s="87"/>
-      <c r="C24" s="88" t="s">
+      <c r="B24" s="40"/>
+      <c r="C24" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="D24" s="89"/>
-      <c r="E24" s="89" t="s">
+      <c r="D24" s="42"/>
+      <c r="E24" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="F24" s="90"/>
+      <c r="F24" s="43"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
@@ -1710,13 +1743,21 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A8:C12"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="D16:E16"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="A1:E2"/>
     <mergeCell ref="A3:B3"/>
@@ -1726,27 +1767,20 @@
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="A8:C12"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
-  <webPublishItems count="1">
+  <webPublishItems count="2">
     <webPublishItem id="25943" divId="payment_order_25943" sourceType="range" sourceRef="A1:F27" destinationFile="C:\Users\Mariano\Desktop\payment_order.htm"/>
+    <webPublishItem id="10753" divId="payment_order_10753" sourceType="range" sourceRef="A1:F27" destinationFile="D:\Proyectos\uta-gestion-ops\templates\payment_order\payment_order.htm"/>
   </webPublishItems>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: fixed account name format
</commit_message>
<xml_diff>
--- a/templates/payment_order/payment_order.xlsx
+++ b/templates/payment_order/payment_order.xlsx
@@ -134,44 +134,44 @@
 PABLO</t>
   </si>
   <si>
+    <t>{{ paymnet_order_id }}</t>
+  </si>
+  <si>
+    <t>{{ payment_order_date }}</t>
+  </si>
+  <si>
+    <t>{{ supplier_name }}</t>
+  </si>
+  <si>
+    <t>{{ invoice_amount }}</t>
+  </si>
+  <si>
+    <t>{{ detail }}</t>
+  </si>
+  <si>
+    <t>{{ witholding_amount }}</t>
+  </si>
+  <si>
+    <t>{{ payment_order_total }}</t>
+  </si>
+  <si>
+    <t>{{ invoice_number }}</t>
+  </si>
+  <si>
+    <t>{{ account_number }}</t>
+  </si>
+  <si>
+    <t>{{ check_number }}</t>
+  </si>
+  <si>
+    <t>{{ issue_date }}</t>
+  </si>
+  <si>
+    <t>{{ due_date }}</t>
+  </si>
+  <si>
     <t>UNION TRANVIARIOS AUTOMOTOR
-{{ account_name }}</t>
-  </si>
-  <si>
-    <t>{{ paymnet_order_id }}</t>
-  </si>
-  <si>
-    <t>{{ payment_order_date }}</t>
-  </si>
-  <si>
-    <t>{{ supplier_name }}</t>
-  </si>
-  <si>
-    <t>{{ invoice_amount }}</t>
-  </si>
-  <si>
-    <t>{{ detail }}</t>
-  </si>
-  <si>
-    <t>{{ witholding_amount }}</t>
-  </si>
-  <si>
-    <t>{{ payment_order_total }}</t>
-  </si>
-  <si>
-    <t>{{ invoice_number }}</t>
-  </si>
-  <si>
-    <t>{{ account_number }}</t>
-  </si>
-  <si>
-    <t>{{ check_number }}</t>
-  </si>
-  <si>
-    <t>{{ issue_date }}</t>
-  </si>
-  <si>
-    <t>{{ due_date }}</t>
+{{ account_name|upper|join(' ') }}</t>
   </si>
 </sst>
 </file>
@@ -870,49 +870,87 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -969,85 +1007,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1445,71 +1445,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="64" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="65"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="26"/>
+    </row>
+    <row r="2" spans="1:6" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="66"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="69" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="70"/>
+      <c r="C3" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="26"/>
-    </row>
-    <row r="2" spans="1:6" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="52"/>
-      <c r="B2" s="53"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F3" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="72"/>
+      <c r="C4" s="73" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="57" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="59" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="61"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="75"/>
     </row>
     <row r="5" spans="1:6" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="63"/>
-      <c r="C5" s="63"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="38"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="34"/>
     </row>
     <row r="6" spans="1:6" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="66" t="s">
+      <c r="B6" s="79"/>
+      <c r="C6" s="79"/>
+      <c r="D6" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="67"/>
+      <c r="E6" s="81"/>
       <c r="F6" s="8" t="s">
         <v>3</v>
       </c>
@@ -1518,106 +1518,106 @@
       <c r="A7" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="48"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
+      <c r="B7" s="62"/>
+      <c r="C7" s="63"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
       <c r="F7" s="14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="45" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="92" t="s">
+      <c r="B8" s="46"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="15"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="47"/>
+      <c r="B9" s="46"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="15"/>
+    </row>
+    <row r="10" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="47"/>
+      <c r="B10" s="46"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="16"/>
+    </row>
+    <row r="11" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="47"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="16"/>
+    </row>
+    <row r="12" spans="1:6" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="48"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="44"/>
+      <c r="F12" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="93"/>
-      <c r="C8" s="93"/>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="15"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="94"/>
-      <c r="B9" s="93"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="89"/>
-      <c r="E9" s="90"/>
-      <c r="F9" s="15"/>
-    </row>
-    <row r="10" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="94"/>
-      <c r="B10" s="93"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="88"/>
-      <c r="F10" s="16"/>
-    </row>
-    <row r="11" spans="1:6" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="94"/>
-      <c r="B11" s="93"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="88"/>
-      <c r="E11" s="88"/>
-      <c r="F11" s="16"/>
-    </row>
-    <row r="12" spans="1:6" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="95"/>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="91" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="91"/>
-      <c r="F12" s="17" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="33"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="13" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="81" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
     <row r="14" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="82" t="s">
+      <c r="A14" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="83"/>
-      <c r="C14" s="84"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="37"/>
       <c r="D14" s="29"/>
       <c r="E14" s="29"/>
       <c r="F14" s="24"/>
     </row>
     <row r="15" spans="1:6" s="2" customFormat="1" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="73" t="s">
+      <c r="A15" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="74"/>
-      <c r="C15" s="75" t="s">
+      <c r="B15" s="55"/>
+      <c r="C15" s="56" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="57"/>
+      <c r="E15" s="58"/>
+      <c r="F15" s="59"/>
+    </row>
+    <row r="16" spans="1:6" ht="28.35" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="39"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="60" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="61"/>
+      <c r="F16" s="20" t="s">
         <v>40</v>
-      </c>
-      <c r="D15" s="76"/>
-      <c r="E15" s="77"/>
-      <c r="F15" s="78"/>
-    </row>
-    <row r="16" spans="1:6" ht="28.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="85" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="86"/>
-      <c r="C16" s="87"/>
-      <c r="D16" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="E16" s="80"/>
-      <c r="F16" s="20" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1625,32 +1625,32 @@
         <v>22</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" s="21" t="s">
         <v>23</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E17" s="21" t="s">
         <v>24</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="71" t="s">
+      <c r="A18" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="72"/>
-      <c r="C18" s="72"/>
-      <c r="D18" s="69" t="s">
+      <c r="B18" s="53"/>
+      <c r="C18" s="53"/>
+      <c r="D18" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="69"/>
-      <c r="F18" s="70"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
     </row>
     <row r="19" spans="1:6" ht="5.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="10"/>
@@ -1664,29 +1664,29 @@
       <c r="A20" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="34"/>
+      <c r="C20" s="84"/>
+      <c r="D20" s="84"/>
+      <c r="E20" s="84"/>
+      <c r="F20" s="85"/>
     </row>
     <row r="21" spans="1:6" ht="62.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="44" t="s">
+      <c r="B21" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="45"/>
+      <c r="C21" s="94"/>
       <c r="D21" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="46" t="s">
+      <c r="E21" s="95" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="47"/>
+      <c r="F21" s="96"/>
     </row>
     <row r="22" spans="1:6" ht="5.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10"/>
@@ -1697,28 +1697,28 @@
       <c r="F22" s="11"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="35" t="s">
+      <c r="A23" s="86" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="36"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="38"/>
+      <c r="B23" s="87"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="34"/>
     </row>
     <row r="24" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="39" t="s">
+      <c r="A24" s="88" t="s">
         <v>5</v>
       </c>
-      <c r="B24" s="40"/>
-      <c r="C24" s="41" t="s">
+      <c r="B24" s="89"/>
+      <c r="C24" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42" t="s">
+      <c r="D24" s="91"/>
+      <c r="E24" s="91" t="s">
         <v>7</v>
       </c>
-      <c r="F24" s="43"/>
+      <c r="F24" s="92"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
@@ -1743,6 +1743,28 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="D16:E16"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A16:C16"/>
@@ -1752,28 +1774,6 @@
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="A8:C12"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="A1:E2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="300" r:id="rId1"/>

</xml_diff>